<commit_message>
config: update endpoints to production web URLs
</commit_message>
<xml_diff>
--- a/WIP_sola.xlsx
+++ b/WIP_sola.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8621715fd65c8d01/Documents/1_PROGRAMMING/2_WEB DEV/1_Products/solanalytica-mvp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\James\OneDrive\Documents\1_PROGRAMMING\2_WEB DEV\1_Products\yieldtrace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10480DE11976A05ADE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D64A6D43-442B-4B55-B9E0-D8FA6103FED5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3ABA55-80CD-41A1-A680-139D2252CE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-1200" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Backlog</t>
   </si>
@@ -147,6 +147,29 @@
   </si>
   <si>
     <t>Formally log the 'Asset Decoupling Audit' as complete in the project management tracker based on successful client-to-backend parameter transmission.</t>
+  </si>
+  <si>
+    <r>
+      <t>Allocate task authorization to deploy the static frontend layer to Netlify with root directory visibility (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) and provision the background Node engine on Render with necessary system environment variables.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -222,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -232,9 +255,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -527,12 +547,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="43.44140625" customWidth="1"/>
-    <col min="2" max="2" width="47.33203125" customWidth="1"/>
-    <col min="3" max="3" width="42.77734375" customWidth="1"/>
-    <col min="4" max="4" width="52.21875" customWidth="1"/>
+    <col min="1" max="1" width="43.42578125" customWidth="1"/>
+    <col min="2" max="2" width="47.28515625" customWidth="1"/>
+    <col min="3" max="3" width="42.7109375" customWidth="1"/>
+    <col min="4" max="4" width="52.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -549,85 +569,86 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="77.400000000000006" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="1:4" ht="77.45" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="67.8" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="7" t="s">
+    <row r="3" spans="1:4" ht="85.5" customHeight="1">
+      <c r="A3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="46.2" customHeight="1">
-      <c r="A4" s="1"/>
+    <row r="4" spans="1:4" ht="46.15" customHeight="1">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="46.2" customHeight="1">
+    <row r="5" spans="1:4" ht="46.15" customHeight="1">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="46.2" customHeight="1">
+    <row r="6" spans="1:4" ht="46.15" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" ht="46.2" customHeight="1">
+    <row r="7" spans="1:4" ht="46.15" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" ht="46.2" customHeight="1">
+    <row r="8" spans="1:4" ht="46.15" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="46.2" customHeight="1">
+    <row r="9" spans="1:4" ht="46.15" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:4" ht="46.2" customHeight="1">
+    <row r="10" spans="1:4" ht="46.15" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4" ht="46.2" customHeight="1">
+    <row r="11" spans="1:4" ht="46.15" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4" ht="46.2" customHeight="1">
+    <row r="12" spans="1:4" ht="46.15" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>

</xml_diff>